<commit_message>
aum script works and excel generated
</commit_message>
<xml_diff>
--- a/scripts/output/managed_aum.xlsx
+++ b/scripts/output/managed_aum.xlsx
@@ -403,7 +403,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Period</v>
       </c>
       <c r="B1" t="str">
         <v>Total AUM</v>
@@ -4286,7 +4286,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Period</v>
       </c>
       <c r="B1" t="str">
         <v>Total AUM</v>
@@ -4294,7 +4294,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2024-03-28</v>
+        <v>Mar 2024</v>
       </c>
       <c r="B2">
         <v>101631879.9713</v>
@@ -4302,7 +4302,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2024-04-30</v>
+        <v>Apr 2024</v>
       </c>
       <c r="B3">
         <v>147312689.7487</v>
@@ -4310,7 +4310,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2024-05-31</v>
+        <v>May 2024</v>
       </c>
       <c r="B4">
         <v>254766939.1165</v>
@@ -4318,7 +4318,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2024-06-28</v>
+        <v>Jun 2024</v>
       </c>
       <c r="B5">
         <v>380602893.1736</v>
@@ -4326,7 +4326,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2024-07-31</v>
+        <v>Jul 2024</v>
       </c>
       <c r="B6">
         <v>369325153.0081</v>
@@ -4334,7 +4334,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2024-08-30</v>
+        <v>Aug 2024</v>
       </c>
       <c r="B7">
         <v>370384405.856</v>
@@ -4342,7 +4342,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2024-09-30</v>
+        <v>Sep 2024</v>
       </c>
       <c r="B8">
         <v>385339039.3109</v>
@@ -4350,7 +4350,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2024-10-31</v>
+        <v>Oct 2024</v>
       </c>
       <c r="B9">
         <v>452485141.2192</v>
@@ -4358,7 +4358,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2024-11-29</v>
+        <v>Nov 2024</v>
       </c>
       <c r="B10">
         <v>579098551.5615</v>
@@ -4366,7 +4366,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2024-12-31</v>
+        <v>Dec 2024</v>
       </c>
       <c r="B11">
         <v>550728392.2268</v>
@@ -4374,7 +4374,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-01-31</v>
+        <v>Jan 2025</v>
       </c>
       <c r="B12">
         <v>558674352.6387</v>
@@ -4382,7 +4382,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-02-28</v>
+        <v>Feb 2025</v>
       </c>
       <c r="B13">
         <v>560796798.5352</v>
@@ -4390,7 +4390,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-03-28</v>
+        <v>Mar 2025</v>
       </c>
       <c r="B14">
         <v>575541898.7093</v>
@@ -4398,7 +4398,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-04-30</v>
+        <v>Apr 2025</v>
       </c>
       <c r="B15">
         <v>800947565.2524</v>
@@ -4406,7 +4406,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-05-30</v>
+        <v>May 2025</v>
       </c>
       <c r="B16">
         <v>896628945.816</v>
@@ -4414,7 +4414,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-06-30</v>
+        <v>Jun 2025</v>
       </c>
       <c r="B17">
         <v>996937807.5971999</v>
@@ -4422,7 +4422,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-07-31</v>
+        <v>Jul 2025</v>
       </c>
       <c r="B18">
         <v>1038350657.2505</v>
@@ -4430,7 +4430,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-08-29</v>
+        <v>Aug 2025</v>
       </c>
       <c r="B19">
         <v>1009172050.6386</v>
@@ -4438,7 +4438,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-09-30</v>
+        <v>Sep 2025</v>
       </c>
       <c r="B20">
         <v>1101813009.4039</v>
@@ -4446,7 +4446,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-10-31</v>
+        <v>Oct 2025</v>
       </c>
       <c r="B21">
         <v>1151168962.5125</v>
@@ -4454,7 +4454,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-28</v>
+        <v>Nov 2025</v>
       </c>
       <c r="B22">
         <v>1478328526.7094002</v>
@@ -4462,7 +4462,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-12-31</v>
+        <v>Dec 2025</v>
       </c>
       <c r="B23">
         <v>1840880601.3631</v>
@@ -4470,7 +4470,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-01-30</v>
+        <v>Jan 2026</v>
       </c>
       <c r="B24">
         <v>2286250343.0716004</v>
@@ -4478,7 +4478,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-02-27</v>
+        <v>Feb 2026</v>
       </c>
       <c r="B25">
         <v>2544523131.2534</v>
@@ -4497,7 +4497,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Date</v>
+        <v>Period</v>
       </c>
       <c r="B1" t="str">
         <v>Total AUM</v>
@@ -4505,7 +4505,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2024-03-28</v>
+        <v>Q1 2024</v>
       </c>
       <c r="B2">
         <v>101631879.9713</v>
@@ -4513,7 +4513,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2024-06-28</v>
+        <v>Q2 2024</v>
       </c>
       <c r="B3">
         <v>380602893.1736</v>
@@ -4521,7 +4521,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2024-09-30</v>
+        <v>Q3 2024</v>
       </c>
       <c r="B4">
         <v>385339039.3109</v>
@@ -4529,7 +4529,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2024-12-31</v>
+        <v>Q4 2024</v>
       </c>
       <c r="B5">
         <v>550728392.2268</v>
@@ -4537,7 +4537,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-03-28</v>
+        <v>Q1 2025</v>
       </c>
       <c r="B6">
         <v>575541898.7093</v>
@@ -4545,7 +4545,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-06-30</v>
+        <v>Q2 2025</v>
       </c>
       <c r="B7">
         <v>996937807.5971999</v>
@@ -4553,7 +4553,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-09-30</v>
+        <v>Q3 2025</v>
       </c>
       <c r="B8">
         <v>1101813009.4039</v>
@@ -4561,7 +4561,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-12-31</v>
+        <v>Q4 2025</v>
       </c>
       <c r="B9">
         <v>1840880601.3631</v>
@@ -4569,7 +4569,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-02-27</v>
+        <v>Q1 2026</v>
       </c>
       <c r="B10">
         <v>2544523131.2534</v>

</xml_diff>